<commit_message>
creates image accessibility alt text.
</commit_message>
<xml_diff>
--- a/spreadsheet_demos/mods_default_basic.xlsx
+++ b/spreadsheet_demos/mods_default_basic.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>identifierFileName</t>
   </si>
@@ -70,6 +70,9 @@
     <t>useAndReproduction</t>
   </si>
   <si>
+    <t>imageAccessibilityAltText</t>
+  </si>
+  <si>
     <t>demo_archival_item_001</t>
   </si>
   <si>
@@ -134,22 +137,17 @@
   </si>
   <si>
     <t>Sparse sample row showing that blank spreadsheet fields are omitted from XML.</t>
+  </si>
+  <si>
+    <t>Front view of a campus building with trees and a walkway.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -164,18 +162,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -189,15 +181,14 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -493,168 +484,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" customWidth="1"/>
-    <col min="16" max="16" width="19.7109375" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" customWidth="1"/>
-    <col min="18" max="18" width="18.7109375" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="R2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="J3" t="s">
+        <v>40</v>
+      </c>
+      <c r="M3" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="N3" t="s">
         <v>31</v>
       </c>
-      <c r="P2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="R2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
-      <c r="A3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="s">
-        <v>30</v>
+      <c r="S3" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>